<commit_message>
feat: Update API test script to handle 422 status codes for negative validations
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="98">
   <si>
     <t>loginName</t>
   </si>
@@ -88,6 +88,9 @@
     <t>12:30 PM</t>
   </si>
   <si>
+    <t>BS-MIRNY-Q6P4N5XGUMULE</t>
+  </si>
+  <si>
     <t>P</t>
   </si>
   <si>
@@ -103,6 +106,9 @@
     <t>Valid Submission (Unit-Based)</t>
   </si>
   <si>
+    <t>06/18/2026</t>
+  </si>
+  <si>
     <t>Happy path units</t>
   </si>
   <si>
@@ -112,6 +118,9 @@
     <t>Missing serviceFormId</t>
   </si>
   <si>
+    <t>06/19/2026</t>
+  </si>
+  <si>
     <t>Missing Form ID</t>
   </si>
   <si>
@@ -124,6 +133,9 @@
     <t>Missing optionCode</t>
   </si>
   <si>
+    <t>06/20/2026</t>
+  </si>
+  <si>
     <t>Missing option</t>
   </si>
   <si>
@@ -142,6 +154,9 @@
     <t>Invalid Date Format</t>
   </si>
   <si>
+    <t>06/21/2026</t>
+  </si>
+  <si>
     <t>Wrong date format</t>
   </si>
   <si>
@@ -154,6 +169,12 @@
     <t>Non-existent serviceFormId</t>
   </si>
   <si>
+    <t>06/22/2026</t>
+  </si>
+  <si>
+    <t>BS-MIRNY-Q6P4N5XGUMULL</t>
+  </si>
+  <si>
     <t>Fake form ID</t>
   </si>
   <si>
@@ -166,6 +187,9 @@
     <t>Missing Time In/Out when required</t>
   </si>
   <si>
+    <t>06/23/2026</t>
+  </si>
+  <si>
     <t>Time required but missing</t>
   </si>
   <si>
@@ -178,6 +202,9 @@
     <t>Missing Direct Units when required</t>
   </si>
   <si>
+    <t>BS-MIRNY-QBU4MZ9WVMULP</t>
+  </si>
+  <si>
     <t>Units required but missing</t>
   </si>
   <si>
@@ -187,6 +214,9 @@
     <t>Invalid Data Type for Units (String)</t>
   </si>
   <si>
+    <t>06/24/2026</t>
+  </si>
+  <si>
     <t>String instead of number</t>
   </si>
   <si>
@@ -214,6 +244,9 @@
     <t>Submit Negative Units</t>
   </si>
   <si>
+    <t>06/26/2026</t>
+  </si>
+  <si>
     <t>Negative value</t>
   </si>
   <si>
@@ -226,6 +259,9 @@
     <t>Exceed Maximum Allowed Units</t>
   </si>
   <si>
+    <t>06/27/2026</t>
+  </si>
+  <si>
     <t>Too large</t>
   </si>
   <si>
@@ -238,6 +274,9 @@
     <t>Units with &gt; 2 Decimal Places</t>
   </si>
   <si>
+    <t>06/28/2026</t>
+  </si>
+  <si>
     <t>3 decimals</t>
   </si>
   <si>
@@ -250,6 +289,9 @@
     <t>Time In is later than Time Out</t>
   </si>
   <si>
+    <t>06/29/2026</t>
+  </si>
+  <si>
     <t>02:30 PM</t>
   </si>
   <si>
@@ -265,58 +307,13 @@
     <t>Approval without Time Out</t>
   </si>
   <si>
+    <t>06/30/2026</t>
+  </si>
+  <si>
     <t>Missing timeout on approval</t>
   </si>
   <si>
     <t>Time Out is required when Time In is provided to ‘Approve’ attendance</t>
-  </si>
-  <si>
-    <t>BS-MIRNY-Q6P4N5XGUMULE</t>
-  </si>
-  <si>
-    <t>BS-MIRNY-Q6P4N5XGUMULL</t>
-  </si>
-  <si>
-    <t>BS-MIRNY-QBU4MZ9WVMULP</t>
-  </si>
-  <si>
-    <t>06/01/2026</t>
-  </si>
-  <si>
-    <t>06/02/2026</t>
-  </si>
-  <si>
-    <t>06/03/2026</t>
-  </si>
-  <si>
-    <t>06/04/2026</t>
-  </si>
-  <si>
-    <t>06/05/2026</t>
-  </si>
-  <si>
-    <t>06/06/2026</t>
-  </si>
-  <si>
-    <t>06/07/2026</t>
-  </si>
-  <si>
-    <t>06/08/2026</t>
-  </si>
-  <si>
-    <t>06/10/2026</t>
-  </si>
-  <si>
-    <t>06/11/2026</t>
-  </si>
-  <si>
-    <t>06/12/2026</t>
-  </si>
-  <si>
-    <t>06/13/2026</t>
-  </si>
-  <si>
-    <t>06/14/2026</t>
   </si>
 </sst>
 </file>
@@ -354,7 +351,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -698,9 +695,8 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="30.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="24.33203125" customWidth="1"/>
-    <col min="8" max="8" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="25.25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -711,7 +707,7 @@
       <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>8</v>
       </c>
       <c r="D1" t="s">
@@ -749,8 +745,8 @@
       <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>86</v>
+      <c r="C2" s="1">
+        <v>46190</v>
       </c>
       <c r="D2" t="s">
         <v>20</v>
@@ -759,16 +755,16 @@
         <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J2">
         <v>200</v>
@@ -776,25 +772,25 @@
     </row>
     <row r="3" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>87</v>
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
       </c>
       <c r="F3" t="s">
-        <v>83</v>
+        <v>60</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J3">
         <v>200</v>
@@ -805,13 +801,13 @@
     </row>
     <row r="4" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>88</v>
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
       </c>
       <c r="D4" t="s">
         <v>20</v>
@@ -820,30 +816,30 @@
         <v>21</v>
       </c>
       <c r="G4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I4" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="J4">
         <v>400</v>
       </c>
       <c r="L4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>89</v>
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
       </c>
       <c r="D5" t="s">
         <v>20</v>
@@ -852,27 +848,27 @@
         <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="H5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J5">
+        <v>400</v>
+      </c>
+      <c r="L5" t="s">
         <v>34</v>
-      </c>
-      <c r="J5">
-        <v>400</v>
-      </c>
-      <c r="L5" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
@@ -881,33 +877,33 @@
         <v>21</v>
       </c>
       <c r="F6" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="J6">
         <v>400</v>
       </c>
       <c r="L6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>90</v>
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
       </c>
       <c r="D7" t="s">
         <v>20</v>
@@ -916,33 +912,33 @@
         <v>21</v>
       </c>
       <c r="F7" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I7" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="J7">
         <v>400</v>
       </c>
       <c r="L7" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>91</v>
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
@@ -951,123 +947,123 @@
         <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>84</v>
+        <v>50</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I8" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="J8">
         <v>400</v>
       </c>
       <c r="L8" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>92</v>
+        <v>54</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
       </c>
       <c r="F9" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I9" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="J9">
         <v>400</v>
       </c>
       <c r="L9" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="B10" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>92</v>
+        <v>59</v>
+      </c>
+      <c r="C10" t="s">
+        <v>55</v>
       </c>
       <c r="F10" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I10" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="J10">
         <v>400</v>
       </c>
       <c r="L10" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
       <c r="B11" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
+      </c>
+      <c r="C11" t="s">
+        <v>64</v>
       </c>
       <c r="F11" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="J11">
         <v>400</v>
       </c>
       <c r="K11" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="L11" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>93</v>
+        <v>69</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
       </c>
       <c r="D12" t="s">
         <v>20</v>
@@ -1076,45 +1072,45 @@
         <v>21</v>
       </c>
       <c r="F12" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G12" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I12" t="s">
-        <v>60</v>
+        <v>70</v>
       </c>
       <c r="J12">
         <v>400</v>
       </c>
       <c r="L12" t="s">
-        <v>61</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>94</v>
+        <v>73</v>
+      </c>
+      <c r="C13" t="s">
+        <v>74</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="G13" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I13" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="J13">
         <v>400</v>
@@ -1123,30 +1119,30 @@
         <v>-2</v>
       </c>
       <c r="L13" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>66</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>67</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>95</v>
+        <v>78</v>
+      </c>
+      <c r="C14" t="s">
+        <v>79</v>
       </c>
       <c r="F14" t="s">
-        <v>85</v>
+        <v>60</v>
       </c>
       <c r="G14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I14" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="J14">
         <v>400</v>
@@ -1155,30 +1151,30 @@
         <v>100000000</v>
       </c>
       <c r="L14" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
     </row>
     <row r="15" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>96</v>
+        <v>83</v>
+      </c>
+      <c r="C15" t="s">
+        <v>84</v>
       </c>
       <c r="F15" t="s">
+        <v>60</v>
+      </c>
+      <c r="G15" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I15" t="s">
         <v>85</v>
-      </c>
-      <c r="G15" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15" t="s">
-        <v>72</v>
       </c>
       <c r="J15">
         <v>400</v>
@@ -1187,81 +1183,80 @@
         <v>4.125</v>
       </c>
       <c r="L15" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>97</v>
+        <v>88</v>
+      </c>
+      <c r="C16" t="s">
+        <v>89</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>90</v>
       </c>
       <c r="E16" t="s">
         <v>20</v>
       </c>
       <c r="F16" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G16" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I16" t="s">
-        <v>77</v>
+        <v>91</v>
       </c>
       <c r="J16">
         <v>400</v>
       </c>
       <c r="L16" t="s">
-        <v>78</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>79</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>98</v>
+        <v>94</v>
+      </c>
+      <c r="C17" t="s">
+        <v>95</v>
       </c>
       <c r="D17" t="s">
         <v>20</v>
       </c>
       <c r="F17" t="s">
-        <v>83</v>
+        <v>22</v>
       </c>
       <c r="G17" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I17" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="J17">
         <v>400</v>
       </c>
       <c r="L17" t="s">
-        <v>82</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L1 A4:B4 A2:B2 G2:L2 A3:B3 G3:L3 A12:B12 A5:B5 G5:L5 A6:E6 G6:L6 A7:B7 G7:L7 A8:B8 G8:L8 A9:B9 G9:L9 A10:B10 G10:L10 A11:B11 G11:L11 A17:B17 A13:B13 G13:L13 A14:B14 G14:L14 A15:B15 G15:L15 A16:B16 G16:L16 G17:L17 D2:E2 D3:E3 D4:L4 D5:E5 D7:E7 D8:E8 D9:E9 D10:E10 D11:E11 D12:E12 D13:E13 D14:E14 D15:E15 D16:E16 D17:E17 G12:L12" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L1 A4:L17 A3:E3 G3:L3 A2:B2 D2:L2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated the excel file
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -2,14 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MirzaMehediIqbal\Desktop\Therap_API_Automation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Att_Api_automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7190" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23820" windowHeight="9765" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Credentials" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="101">
   <si>
     <t>loginName</t>
   </si>
@@ -106,7 +106,7 @@
     <t>Valid Submission (Unit-Based)</t>
   </si>
   <si>
-    <t>06/18/2026</t>
+    <t>BS-MIRNY-QBU4MZ9WVMULP</t>
   </si>
   <si>
     <t>Happy path units</t>
@@ -118,9 +118,6 @@
     <t>Missing serviceFormId</t>
   </si>
   <si>
-    <t>06/19/2026</t>
-  </si>
-  <si>
     <t>Missing Form ID</t>
   </si>
   <si>
@@ -133,9 +130,6 @@
     <t>Missing optionCode</t>
   </si>
   <si>
-    <t>06/20/2026</t>
-  </si>
-  <si>
     <t>Missing option</t>
   </si>
   <si>
@@ -154,9 +148,6 @@
     <t>Invalid Date Format</t>
   </si>
   <si>
-    <t>06/21/2026</t>
-  </si>
-  <si>
     <t>Wrong date format</t>
   </si>
   <si>
@@ -169,9 +160,6 @@
     <t>Non-existent serviceFormId</t>
   </si>
   <si>
-    <t>06/22/2026</t>
-  </si>
-  <si>
     <t>BS-MIRNY-Q6P4N5XGUMULL</t>
   </si>
   <si>
@@ -187,9 +175,6 @@
     <t>Missing Time In/Out when required</t>
   </si>
   <si>
-    <t>06/23/2026</t>
-  </si>
-  <si>
     <t>Time required but missing</t>
   </si>
   <si>
@@ -202,9 +187,6 @@
     <t>Missing Direct Units when required</t>
   </si>
   <si>
-    <t>BS-MIRNY-QBU4MZ9WVMULP</t>
-  </si>
-  <si>
     <t>Units required but missing</t>
   </si>
   <si>
@@ -214,9 +196,6 @@
     <t>Invalid Data Type for Units (String)</t>
   </si>
   <si>
-    <t>06/24/2026</t>
-  </si>
-  <si>
     <t>String instead of number</t>
   </si>
   <si>
@@ -244,9 +223,6 @@
     <t>Submit Negative Units</t>
   </si>
   <si>
-    <t>06/26/2026</t>
-  </si>
-  <si>
     <t>Negative value</t>
   </si>
   <si>
@@ -259,9 +235,6 @@
     <t>Exceed Maximum Allowed Units</t>
   </si>
   <si>
-    <t>06/27/2026</t>
-  </si>
-  <si>
     <t>Too large</t>
   </si>
   <si>
@@ -274,9 +247,6 @@
     <t>Units with &gt; 2 Decimal Places</t>
   </si>
   <si>
-    <t>06/28/2026</t>
-  </si>
-  <si>
     <t>3 decimals</t>
   </si>
   <si>
@@ -289,9 +259,6 @@
     <t>Time In is later than Time Out</t>
   </si>
   <si>
-    <t>06/29/2026</t>
-  </si>
-  <si>
     <t>02:30 PM</t>
   </si>
   <si>
@@ -307,13 +274,55 @@
     <t>Approval without Time Out</t>
   </si>
   <si>
-    <t>06/30/2026</t>
-  </si>
-  <si>
     <t>Missing timeout on approval</t>
   </si>
   <si>
     <t>Time Out is required when Time In is provided to ‘Approve’ attendance</t>
+  </si>
+  <si>
+    <t>08/01/2026</t>
+  </si>
+  <si>
+    <t>08/02/2026</t>
+  </si>
+  <si>
+    <t>08/03/2026</t>
+  </si>
+  <si>
+    <t>08/04/2026</t>
+  </si>
+  <si>
+    <t>08/05/2026</t>
+  </si>
+  <si>
+    <t>08/06/2026</t>
+  </si>
+  <si>
+    <t>08/07/2026</t>
+  </si>
+  <si>
+    <t>08/08/2026</t>
+  </si>
+  <si>
+    <t>08/09/2026</t>
+  </si>
+  <si>
+    <t>08/10/2026</t>
+  </si>
+  <si>
+    <t>08/11/2026</t>
+  </si>
+  <si>
+    <t>08/12/2026</t>
+  </si>
+  <si>
+    <t>08/13/2026</t>
+  </si>
+  <si>
+    <t>08/14/2026</t>
+  </si>
+  <si>
+    <t>08/15/2026</t>
   </si>
 </sst>
 </file>
@@ -351,7 +360,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,7 +421,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -447,7 +456,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -514,20 +523,16 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="100000"/>
+                <a:shade val="100000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
+                <a:tint val="50000"/>
+                <a:shade val="100000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -649,7 +654,46 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
   <a:extraClrSchemeLst/>
 </a:theme>
 </file>
@@ -657,9 +701,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -670,7 +714,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -692,22 +736,29 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="11.125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="26" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="8.625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="26.125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.25" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="59.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>6</v>
       </c>
       <c r="B1" t="s">
         <v>7</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="D1" t="s">
@@ -738,15 +789,15 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
       <c r="B2" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="1">
-        <v>46190</v>
+      <c r="C2" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="D2" t="s">
         <v>20</v>
@@ -770,18 +821,18 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>26</v>
       </c>
       <c r="B3" t="s">
         <v>27</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F3" t="s">
         <v>28</v>
-      </c>
-      <c r="F3" t="s">
-        <v>60</v>
       </c>
       <c r="G3" t="s">
         <v>23</v>
@@ -799,15 +850,15 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
       <c r="B4" t="s">
         <v>31</v>
       </c>
-      <c r="C4" t="s">
-        <v>32</v>
+      <c r="C4" s="1" t="s">
+        <v>88</v>
       </c>
       <c r="D4" t="s">
         <v>20</v>
@@ -822,24 +873,24 @@
         <v>24</v>
       </c>
       <c r="I4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J4">
         <v>400</v>
       </c>
       <c r="L4" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C5" t="s">
-        <v>37</v>
+      <c r="C5" s="1" t="s">
+        <v>89</v>
       </c>
       <c r="D5" t="s">
         <v>20</v>
@@ -854,21 +905,24 @@
         <v>24</v>
       </c>
       <c r="I5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J5">
         <v>400</v>
       </c>
       <c r="L5" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="D6" t="s">
         <v>20</v>
@@ -886,24 +940,24 @@
         <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="J6">
         <v>400</v>
       </c>
       <c r="L6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
-      </c>
-      <c r="C7" t="s">
-        <v>44</v>
+        <v>41</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="D7" t="s">
         <v>20</v>
@@ -921,24 +975,24 @@
         <v>24</v>
       </c>
       <c r="I7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="J7">
         <v>400</v>
       </c>
       <c r="L7" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" t="s">
-        <v>49</v>
+        <v>45</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>92</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
@@ -947,7 +1001,7 @@
         <v>21</v>
       </c>
       <c r="F8" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G8" t="s">
         <v>23</v>
@@ -956,24 +1010,24 @@
         <v>24</v>
       </c>
       <c r="I8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="J8">
         <v>400</v>
       </c>
       <c r="L8" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" t="s">
-        <v>55</v>
+        <v>50</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>93</v>
       </c>
       <c r="F9" t="s">
         <v>22</v>
@@ -985,56 +1039,56 @@
         <v>24</v>
       </c>
       <c r="I9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="J9">
         <v>400</v>
       </c>
       <c r="L9" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="F10" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" t="s">
+        <v>23</v>
+      </c>
+      <c r="H10" t="s">
+        <v>24</v>
+      </c>
+      <c r="I10" t="s">
         <v>55</v>
-      </c>
-      <c r="F10" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" t="s">
-        <v>23</v>
-      </c>
-      <c r="H10" t="s">
-        <v>24</v>
-      </c>
-      <c r="I10" t="s">
-        <v>61</v>
       </c>
       <c r="J10">
         <v>400</v>
       </c>
       <c r="L10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="11" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>62</v>
-      </c>
-      <c r="B11" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" t="s">
-        <v>64</v>
+      <c r="C11" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="G11" t="s">
         <v>23</v>
@@ -1043,27 +1097,27 @@
         <v>24</v>
       </c>
       <c r="I11" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="J11">
         <v>400</v>
       </c>
       <c r="K11" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="L11" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
-      </c>
-      <c r="C12" t="s">
-        <v>64</v>
+        <v>62</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>95</v>
       </c>
       <c r="D12" t="s">
         <v>20</v>
@@ -1081,27 +1135,27 @@
         <v>24</v>
       </c>
       <c r="I12" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="J12">
         <v>400</v>
       </c>
       <c r="L12" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
-      </c>
-      <c r="C13" t="s">
-        <v>74</v>
+        <v>66</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>96</v>
       </c>
       <c r="F13" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="G13" t="s">
         <v>23</v>
@@ -1110,7 +1164,7 @@
         <v>24</v>
       </c>
       <c r="I13" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="J13">
         <v>400</v>
@@ -1119,21 +1173,21 @@
         <v>-2</v>
       </c>
       <c r="L13" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" t="s">
-        <v>79</v>
+        <v>70</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>97</v>
       </c>
       <c r="F14" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="G14" t="s">
         <v>23</v>
@@ -1142,7 +1196,7 @@
         <v>24</v>
       </c>
       <c r="I14" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="J14">
         <v>400</v>
@@ -1151,21 +1205,21 @@
         <v>100000000</v>
       </c>
       <c r="L14" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B15" t="s">
-        <v>83</v>
-      </c>
-      <c r="C15" t="s">
-        <v>84</v>
+        <v>74</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>98</v>
       </c>
       <c r="F15" t="s">
-        <v>60</v>
+        <v>28</v>
       </c>
       <c r="G15" t="s">
         <v>23</v>
@@ -1174,7 +1228,7 @@
         <v>24</v>
       </c>
       <c r="I15" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="J15">
         <v>400</v>
@@ -1183,21 +1237,21 @@
         <v>4.125</v>
       </c>
       <c r="L15" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
-      </c>
-      <c r="C16" t="s">
-        <v>89</v>
+        <v>78</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>99</v>
       </c>
       <c r="D16" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="E16" t="s">
         <v>20</v>
@@ -1212,24 +1266,24 @@
         <v>24</v>
       </c>
       <c r="I16" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="J16">
         <v>400</v>
       </c>
       <c r="L16" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" ht="15.5" x14ac:dyDescent="0.35">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="B17" t="s">
-        <v>94</v>
-      </c>
-      <c r="C17" t="s">
-        <v>95</v>
+        <v>83</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>100</v>
       </c>
       <c r="D17" t="s">
         <v>20</v>
@@ -1244,19 +1298,20 @@
         <v>24</v>
       </c>
       <c r="I17" t="s">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="J17">
         <v>400</v>
       </c>
       <c r="L17" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L1 A4:L17 A3:E3 G3:L3 A2:B2 D2:L2" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:L1 A4:B17 A2:B2 D2:L2 A3:B3 D3:L3 D4:L17" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>